<commit_message>
fix: corrige notebook do dicionário de dados da atividade 02
</commit_message>
<xml_diff>
--- a/dadosBrutos/curriculos.xlsx
+++ b/dadosBrutos/curriculos.xlsx
@@ -2762,6 +2762,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
+    <col customWidth="1" min="1" max="1" width="12.00390625"/>
     <col customWidth="1" min="2" max="2" width="36.140625"/>
   </cols>
   <sheetData>
@@ -2857,7 +2858,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" ht="14.25">
+    <row r="21" ht="51">
       <c r="A21" s="7" t="s">
         <v>16</v>
       </c>
@@ -2877,7 +2878,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" ht="14.25">
+    <row r="22" ht="25.5">
       <c r="A22" s="9" t="s">
         <v>22</v>
       </c>
@@ -2897,7 +2898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="14.25">
+    <row r="23" ht="25.5">
       <c r="A23" s="9" t="s">
         <v>25</v>
       </c>
@@ -2917,7 +2918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" ht="14.25">
+    <row r="24" ht="25.5">
       <c r="A24" s="9" t="s">
         <v>27</v>
       </c>
@@ -2937,7 +2938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="14.25">
+    <row r="25" ht="25.5">
       <c r="A25" s="9" t="s">
         <v>29</v>
       </c>
@@ -2957,7 +2958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" ht="14.25">
+    <row r="26" ht="25.5">
       <c r="A26" s="9" t="s">
         <v>31</v>
       </c>
@@ -2977,7 +2978,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="27" ht="14.25">
+    <row r="27" ht="25.5">
       <c r="A27" s="9" t="s">
         <v>33</v>
       </c>
@@ -2997,7 +2998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" ht="14.25">
+    <row r="28" ht="25.5">
       <c r="A28" s="9" t="s">
         <v>35</v>
       </c>
@@ -3031,7 +3032,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" ht="14.25">
+    <row r="33" ht="51">
       <c r="A33" s="7" t="s">
         <v>16</v>
       </c>
@@ -3251,7 +3252,7 @@
       <c r="E49" s="18"/>
       <c r="F49" s="18"/>
     </row>
-    <row r="50" ht="14.25">
+    <row r="50" ht="25.5">
       <c r="A50" s="9" t="s">
         <v>53</v>
       </c>
@@ -3355,7 +3356,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="60" ht="14.25">
+    <row r="60" ht="51">
       <c r="A60" s="7" t="s">
         <v>16</v>
       </c>
@@ -7372,7 +7373,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="401" ht="51">
+    <row r="401" ht="14.25">
       <c r="A401" s="7" t="s">
         <v>16</v>
       </c>
@@ -7584,7 +7585,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="420" ht="51">
+    <row r="420" ht="14.25">
       <c r="A420" s="7" t="s">
         <v>16</v>
       </c>

</xml_diff>